<commit_message>
Name the xlsx source column SOURCE_i, reading DOCUMENT_i as before
SOURCE_i takes a document or a unit id and the importer resolves the kind
from the id. DOCUMENT_i is still read, as SOURCE_i, never lost; the
exporter, the template and the StratiMiner prompt write SOURCE_i.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/s3dgraphy/templates/em_data_template.xlsx
+++ b/src/s3dgraphy/templates/em_data_template.xlsx
@@ -786,7 +786,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>DOCUMENT_1</t>
+          <t>SOURCE_1</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>DOCUMENT_2</t>
+          <t>SOURCE_2</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">

</xml_diff>